<commit_message>
Estoque atualizado - 23/03/2026 09:49
</commit_message>
<xml_diff>
--- a/estoque_andamento.xlsx
+++ b/estoque_andamento.xlsx
@@ -1063,9 +1063,9 @@
       <c r="J9" s="4" t="n">
         <v>46098</v>
       </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1447,9 +1447,9 @@
       <c r="J15" s="4" t="n">
         <v>46093</v>
       </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1639,9 +1639,9 @@
       <c r="J18" s="4" t="n">
         <v>46091</v>
       </c>
-      <c r="K18" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2087,9 +2087,9 @@
       <c r="J25" s="4" t="n">
         <v>46097</v>
       </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2215,9 +2215,9 @@
       <c r="J27" s="4" t="n">
         <v>46090</v>
       </c>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2855,9 +2855,9 @@
       <c r="J37" s="4" t="n">
         <v>46085</v>
       </c>
-      <c r="K37" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3431,9 +3431,9 @@
       <c r="J46" s="4" t="n">
         <v>46052</v>
       </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
@@ -3478,12 +3478,12 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Confecção de documentos</t>
+          <t>Assinatura</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Escritura de cessão</t>
+          <t>Assinaturas no cartório</t>
         </is>
       </c>
       <c r="H47" s="3" t="n">
@@ -3623,9 +3623,9 @@
       <c r="J49" s="4" t="n">
         <v>46094</v>
       </c>
-      <c r="K49" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
@@ -3751,9 +3751,9 @@
       <c r="J51" s="4" t="n">
         <v>46092</v>
       </c>
-      <c r="K51" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
@@ -3798,12 +3798,12 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Conferência final</t>
+          <t>Parecer jurídico</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Conferência final</t>
+          <t>Parecer jurídico</t>
         </is>
       </c>
       <c r="H52" s="3" t="n">
@@ -3815,9 +3815,9 @@
       <c r="J52" s="4" t="n">
         <v>46092</v>
       </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -4071,9 +4071,9 @@
       <c r="J56" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K56" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K56" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
@@ -4455,9 +4455,9 @@
       <c r="J62" s="4" t="n">
         <v>46100</v>
       </c>
-      <c r="K62" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K62" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
@@ -4711,9 +4711,9 @@
       <c r="J66" s="4" t="n">
         <v>46092</v>
       </c>
-      <c r="K66" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Análise do ativo - Análise do cedente</t>
+          <t>Emissão de CND Complementares</t>
         </is>
       </c>
       <c r="H67" s="3" t="n">
@@ -5031,9 +5031,9 @@
       <c r="J71" s="4" t="n">
         <v>46085</v>
       </c>
-      <c r="K71" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Análise do ativo - Estudo do processo judicial</t>
+          <t>Análise do ativo - Advogados</t>
         </is>
       </c>
       <c r="H74" s="3" t="n">
@@ -5415,9 +5415,9 @@
       <c r="J77" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K77" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
@@ -5479,9 +5479,9 @@
       <c r="J78" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K78" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
@@ -5863,9 +5863,9 @@
       <c r="J84" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K84" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L84" s="2" t="inlineStr">
@@ -5991,9 +5991,9 @@
       <c r="J86" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K86" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K86" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
@@ -6311,9 +6311,9 @@
       <c r="J91" s="4" t="n">
         <v>46084</v>
       </c>
-      <c r="K91" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L91" s="2" t="inlineStr">
@@ -6503,9 +6503,9 @@
       <c r="J94" s="4" t="n">
         <v>46097</v>
       </c>
-      <c r="K94" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr">
@@ -6567,9 +6567,9 @@
       <c r="J95" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K95" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K95" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr">
@@ -6951,9 +6951,9 @@
       <c r="J101" s="4" t="n">
         <v>46094</v>
       </c>
-      <c r="K101" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L101" s="2" t="inlineStr">
@@ -7126,12 +7126,12 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Parecer jurídico</t>
+          <t>Confecção de documentos</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Parecer jurídico</t>
+          <t>Escritura de cessão</t>
         </is>
       </c>
       <c r="H104" s="3" t="n">
@@ -7207,9 +7207,9 @@
       <c r="J105" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K105" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K105" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L105" s="2" t="inlineStr">
@@ -7446,12 +7446,12 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>Assinatura</t>
+          <t>Protocolo de cessão</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Assinaturas no cartório</t>
+          <t>Protocolo de cessão</t>
         </is>
       </c>
       <c r="H109" s="3" t="n">
@@ -7655,9 +7655,9 @@
       <c r="J112" s="4" t="n">
         <v>46079</v>
       </c>
-      <c r="K112" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L112" s="2" t="inlineStr">
@@ -8099,9 +8099,9 @@
       <c r="J119" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K119" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K119" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L119" s="2" t="inlineStr">
@@ -8547,9 +8547,9 @@
       <c r="J126" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K126" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L126" s="2" t="inlineStr">
@@ -8611,9 +8611,9 @@
       <c r="J127" s="4" t="n">
         <v>46100</v>
       </c>
-      <c r="K127" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K127" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L127" s="2" t="inlineStr">
@@ -8675,9 +8675,9 @@
       <c r="J128" s="4" t="n">
         <v>46091</v>
       </c>
-      <c r="K128" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L128" s="2" t="inlineStr">
@@ -8803,9 +8803,9 @@
       <c r="J130" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K130" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L130" s="2" t="inlineStr">
@@ -9059,9 +9059,9 @@
       <c r="J134" s="4" t="n">
         <v>46100</v>
       </c>
-      <c r="K134" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L134" s="2" t="inlineStr">
@@ -9187,9 +9187,9 @@
       <c r="J136" s="4" t="n">
         <v>46094</v>
       </c>
-      <c r="K136" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L136" s="2" t="inlineStr">
@@ -9251,9 +9251,9 @@
       <c r="J137" s="4" t="n">
         <v>46090</v>
       </c>
-      <c r="K137" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L137" s="2" t="inlineStr">
@@ -9315,9 +9315,9 @@
       <c r="J138" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K138" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L138" s="2" t="inlineStr">
@@ -9426,12 +9426,12 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>Conferência final</t>
+          <t>Parecer jurídico</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>Conferência final</t>
+          <t>Parecer jurídico</t>
         </is>
       </c>
       <c r="H140" s="3" t="n">
@@ -9571,9 +9571,9 @@
       <c r="J142" s="4" t="n">
         <v>46100</v>
       </c>
-      <c r="K142" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L142" s="2" t="inlineStr">
@@ -9891,9 +9891,9 @@
       <c r="J147" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K147" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L147" s="2" t="inlineStr">
@@ -10574,10 +10574,10 @@
         <v>28179814.82</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.2318840579710145</v>
       </c>
       <c r="H2" s="6" t="n">
         <v>2911512.17</v>
@@ -10604,10 +10604,10 @@
         <v>9447668.310000001</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>0.4418604651162791</v>
+        <v>0.3953488372093023</v>
       </c>
       <c r="H3" s="6" t="n">
         <v>1047728.8</v>
@@ -10634,10 +10634,10 @@
         <v>9466694.93</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>0.3076923076923077</v>
+        <v>0.2307692307692308</v>
       </c>
       <c r="H4" s="6" t="n">
         <v>1814883.3</v>
@@ -10664,10 +10664,10 @@
         <v>5514339.61</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.4</v>
+        <v>0.1666666666666666</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>393749.8</v>
@@ -10690,10 +10690,10 @@
         <v>52608517.67</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.3741935483870968</v>
+        <v>0.2645161290322581</v>
       </c>
       <c r="H6" s="8" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Estoque atualizado - 23/03/2026 10:08
</commit_message>
<xml_diff>
--- a/estoque_andamento.xlsx
+++ b/estoque_andamento.xlsx
@@ -1063,9 +1063,9 @@
       <c r="J9" s="4" t="n">
         <v>46098</v>
       </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1447,9 +1447,9 @@
       <c r="J15" s="4" t="n">
         <v>46093</v>
       </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1639,9 +1639,9 @@
       <c r="J18" s="4" t="n">
         <v>46091</v>
       </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2087,9 +2087,9 @@
       <c r="J25" s="4" t="n">
         <v>46097</v>
       </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2215,9 +2215,9 @@
       <c r="J27" s="4" t="n">
         <v>46090</v>
       </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2855,9 +2855,9 @@
       <c r="J37" s="4" t="n">
         <v>46085</v>
       </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3431,9 +3431,9 @@
       <c r="J46" s="4" t="n">
         <v>46052</v>
       </c>
-      <c r="K46" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
@@ -3623,9 +3623,9 @@
       <c r="J49" s="4" t="n">
         <v>46094</v>
       </c>
-      <c r="K49" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
@@ -3751,9 +3751,9 @@
       <c r="J51" s="4" t="n">
         <v>46092</v>
       </c>
-      <c r="K51" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
@@ -3815,9 +3815,9 @@
       <c r="J52" s="4" t="n">
         <v>46092</v>
       </c>
-      <c r="K52" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -4071,9 +4071,9 @@
       <c r="J56" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K56" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
@@ -4455,9 +4455,9 @@
       <c r="J62" s="4" t="n">
         <v>46100</v>
       </c>
-      <c r="K62" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
@@ -4711,9 +4711,9 @@
       <c r="J66" s="4" t="n">
         <v>46092</v>
       </c>
-      <c r="K66" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K66" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
@@ -5031,9 +5031,9 @@
       <c r="J71" s="4" t="n">
         <v>46085</v>
       </c>
-      <c r="K71" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K71" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
@@ -5415,9 +5415,9 @@
       <c r="J77" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K77" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K77" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
@@ -5863,9 +5863,9 @@
       <c r="J84" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K84" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K84" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L84" s="2" t="inlineStr">
@@ -5991,9 +5991,9 @@
       <c r="J86" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K86" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K86" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
@@ -6311,9 +6311,9 @@
       <c r="J91" s="4" t="n">
         <v>46084</v>
       </c>
-      <c r="K91" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K91" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L91" s="2" t="inlineStr">
@@ -6503,9 +6503,9 @@
       <c r="J94" s="4" t="n">
         <v>46097</v>
       </c>
-      <c r="K94" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K94" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr">
@@ -6567,9 +6567,9 @@
       <c r="J95" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K95" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K95" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr">
@@ -6951,9 +6951,9 @@
       <c r="J101" s="4" t="n">
         <v>46094</v>
       </c>
-      <c r="K101" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K101" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L101" s="2" t="inlineStr">
@@ -7207,9 +7207,9 @@
       <c r="J105" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K105" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K105" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L105" s="2" t="inlineStr">
@@ -7655,9 +7655,9 @@
       <c r="J112" s="4" t="n">
         <v>46079</v>
       </c>
-      <c r="K112" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K112" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L112" s="2" t="inlineStr">
@@ -8099,9 +8099,9 @@
       <c r="J119" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K119" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K119" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L119" s="2" t="inlineStr">
@@ -8547,9 +8547,9 @@
       <c r="J126" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K126" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K126" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L126" s="2" t="inlineStr">
@@ -8611,9 +8611,9 @@
       <c r="J127" s="4" t="n">
         <v>46100</v>
       </c>
-      <c r="K127" s="5" t="inlineStr">
-        <is>
-          <t>Sim</t>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
       <c r="L127" s="2" t="inlineStr">
@@ -8675,9 +8675,9 @@
       <c r="J128" s="4" t="n">
         <v>46091</v>
       </c>
-      <c r="K128" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K128" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L128" s="2" t="inlineStr">
@@ -8803,9 +8803,9 @@
       <c r="J130" s="4" t="n">
         <v>46099</v>
       </c>
-      <c r="K130" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K130" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L130" s="2" t="inlineStr">
@@ -9059,9 +9059,9 @@
       <c r="J134" s="4" t="n">
         <v>46100</v>
       </c>
-      <c r="K134" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K134" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L134" s="2" t="inlineStr">
@@ -9187,9 +9187,9 @@
       <c r="J136" s="4" t="n">
         <v>46094</v>
       </c>
-      <c r="K136" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K136" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L136" s="2" t="inlineStr">
@@ -9251,9 +9251,9 @@
       <c r="J137" s="4" t="n">
         <v>46090</v>
       </c>
-      <c r="K137" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K137" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L137" s="2" t="inlineStr">
@@ -9315,9 +9315,9 @@
       <c r="J138" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K138" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K138" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L138" s="2" t="inlineStr">
@@ -9571,9 +9571,9 @@
       <c r="J142" s="4" t="n">
         <v>46100</v>
       </c>
-      <c r="K142" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K142" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L142" s="2" t="inlineStr">
@@ -9891,9 +9891,9 @@
       <c r="J147" s="4" t="n">
         <v>46101</v>
       </c>
-      <c r="K147" s="2" t="inlineStr">
-        <is>
-          <t>Não</t>
+      <c r="K147" s="5" t="inlineStr">
+        <is>
+          <t>Sim</t>
         </is>
       </c>
       <c r="L147" s="2" t="inlineStr">
@@ -10574,10 +10574,10 @@
         <v>28179814.82</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>0.2318840579710145</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H2" s="6" t="n">
         <v>2911512.17</v>
@@ -10604,10 +10604,10 @@
         <v>9447668.310000001</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>0.3953488372093023</v>
+        <v>0.4186046511627907</v>
       </c>
       <c r="H3" s="6" t="n">
         <v>1047728.8</v>
@@ -10634,10 +10634,10 @@
         <v>9466694.93</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>0.2307692307692308</v>
+        <v>0.3076923076923077</v>
       </c>
       <c r="H4" s="6" t="n">
         <v>1814883.3</v>
@@ -10664,10 +10664,10 @@
         <v>5514339.61</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.1666666666666666</v>
+        <v>0.4</v>
       </c>
       <c r="H5" s="6" t="n">
         <v>393749.8</v>
@@ -10690,10 +10690,10 @@
         <v>52608517.67</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.2645161290322581</v>
+        <v>0.367741935483871</v>
       </c>
       <c r="H6" s="8" t="inlineStr"/>
     </row>

</xml_diff>